<commit_message>
AIRARABIA corrected on the growth-basis error
Its terminal was handed a profit figure, a depreciation charge and a working
capital balance all already grown by (1+g), which the sanctioned construction
grows again. On a name whose terminal is 96% OF ENTERPRISE VALUE that is
nearly the whole error.

Central 4.8511 -> 4.7459, gap -2.4% -> -4.5%, still inside the band so no
review is owed. The terminal lever reads 4.2948 corrected, against the 4.39 it
carried, and the route is 4.1745 -> 4.2948 -> 4.7171 -> 4.7459.

All three of its scenario paths carried the same error and all three are
corrected, not just the headline call.

Study checks: recalc 663 of 663 formula cells with 49 headline
reconciliations, 32 drivers, 28 tables 0 unreconciled, 313 prose figures 0
unmatched.

Three studies remain: EMPOWER, DU, MODON.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017RcjXG4ETjADcoFJf123yY
</commit_message>
<xml_diff>
--- a/engine/airarabia_study/AIRARABIA_Valuation_Model_09082026_public.xlsx
+++ b/engine/airarabia_study/AIRARABIA_Valuation_Model_09082026_public.xlsx
@@ -2765,19 +2765,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>6.613931971702153</v>
+        <v>6.530864632088698</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>7.22938797416904</v>
+        <v>7.102168803376595</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>8.047303999567715</v>
+        <v>7.860833702331569</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>9.189336112633173</v>
+        <v>8.919442388482089</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>10.88022997212353</v>
+        <v>10.48530965071819</v>
       </c>
     </row>
     <row r="7">
@@ -2787,19 +2787,19 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>5.290650036151688</v>
+        <v>5.22620977758266</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>5.628038240398886</v>
+        <v>5.532093014962125</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>6.047709804384486</v>
+        <v>5.912111496029038</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>6.584966343990367</v>
+        <v>6.398071091427047</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>7.298672947301888</v>
+        <v>7.043007769349051</v>
       </c>
     </row>
     <row r="8">
@@ -2809,19 +2809,19 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>4.411265519707568</v>
+        <v>4.359176372904554</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>4.611970399626963</v>
+        <v>4.535826864943507</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>4.851184061604538</v>
+        <v>4.745966396016637</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>5.14175332927026</v>
+        <v>5.000767165165692</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>5.502954385226047</v>
+        <v>5.316992642879297</v>
       </c>
     </row>
     <row r="9">
@@ -2831,19 +2831,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>3.785338160707695</v>
+        <v>3.742017746254053</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>3.910801948149978</v>
+        <v>3.848289311017446</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>4.055845559017758</v>
+        <v>3.970774028444986</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4.225812539903896</v>
+        <v>4.113896644092114</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4.428185438899458</v>
+        <v>4.283853112430982</v>
       </c>
     </row>
     <row r="10">
@@ -2853,19 +2853,19 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>3.317696432266285</v>
+        <v>3.280908427380842</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>3.398430090879895</v>
+        <v>3.345850013323994</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>3.489585452220582</v>
+        <v>3.418818015716527</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.593568894394453</v>
+        <v>3.501665739466495</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>3.713589416492556</v>
+        <v>3.596864638976781</v>
       </c>
     </row>
     <row r="12">
@@ -2914,19 +2914,19 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>8.190595518800578</v>
+        <v>8.000623234748355</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>6.152900095652542</v>
+        <v>6.014763569019446</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>4.933557898331902</v>
+        <v>4.826377818105075</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>4.12305166807534</v>
+        <v>4.036399438767721</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>3.545995708484645</v>
+        <v>3.473918397822978</v>
       </c>
     </row>
     <row r="15">
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>8.118262350506111</v>
+        <v>7.930067114029304</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>6.099847501414335</v>
+        <v>5.962997828691612</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>4.89203512682659</v>
+        <v>4.785849443207093</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>4.089186917413269</v>
+        <v>4.003335375343121</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>3.517578411938233</v>
+        <v>3.446164434809923</v>
       </c>
     </row>
     <row r="16">
@@ -2958,19 +2958,19 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>8.046922852356397</v>
+        <v>7.860480281412786</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>6.047521370368907</v>
+        <v>5.911940959735956</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>4.851079136958488</v>
+        <v>4.745874305379804</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>4.055782974525162</v>
+        <v>3.970721252795083</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>3.489546608836069</v>
+        <v>3.418786994571136</v>
       </c>
     </row>
     <row r="17">
@@ -2980,19 +2980,19 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>7.976559329993601</v>
+        <v>7.791845476389811</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>5.995908808691096</v>
+        <v>5.861580380242414</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>4.810679901554656</v>
+        <v>4.706442616760781</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>4.022831713053255</v>
+        <v>3.938549136097555</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>3.461893522369199</v>
+        <v>3.391779457697584</v>
       </c>
     </row>
     <row r="18">
@@ -3002,19 +3002,19 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>7.907154453209897</v>
+        <v>7.724145793683983</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>5.944997186851519</v>
+        <v>5.81190376621413</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>4.770827598168174</v>
+        <v>4.667544789338453</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>3.990325171911993</v>
+        <v>3.906811251616137</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>3.434612513025957</v>
+        <v>3.365135338899167</v>
       </c>
     </row>
     <row r="20">
@@ -3059,19 +3059,19 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>5.957451797954994</v>
+        <v>5.824215735162758</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>5.379702321466985</v>
+        <v>5.261113519562423</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>4.851079136958488</v>
+        <v>4.745874305379804</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>4.325720187878041</v>
+        <v>4.233794195992333</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>3.907604314511882</v>
+        <v>3.826225220792922</v>
       </c>
     </row>
     <row r="24">
@@ -3116,19 +3116,19 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>6.443342919647113</v>
+        <v>6.306723155809302</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>5.647211028302799</v>
+        <v>5.526298730594553</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>4.851079136958488</v>
+        <v>4.745874305379804</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>4.054947245614179</v>
+        <v>3.965449880165061</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>3.258815354269865</v>
+        <v>3.18502545495031</v>
       </c>
     </row>
     <row r="28">
@@ -3173,19 +3173,19 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>4.024478047929036</v>
+        <v>3.933010729477441</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>4.437801581315985</v>
+        <v>4.339465506300848</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>4.851079136958488</v>
+        <v>4.745874305379804</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>5.264316942610993</v>
+        <v>5.152243354468767</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>5.677520149872032</v>
+        <v>5.558577805166262</v>
       </c>
     </row>
     <row r="32">
@@ -3230,19 +3230,19 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>2.991805901498502</v>
+        <v>2.922068051995918</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>3.921439448943881</v>
+        <v>3.833968108403248</v>
       </c>
       <c r="D34" s="7" t="n">
-        <v>4.851079136958488</v>
+        <v>4.745874305379804</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>5.780724545348389</v>
+        <v>5.657786222731658</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>6.710375291402692</v>
+        <v>6.569703477747911</v>
       </c>
     </row>
     <row r="36">
@@ -3287,19 +3287,19 @@
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>5.363960992397897</v>
+        <v>5.258756160819213</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>5.107520064678192</v>
+        <v>5.002315233099507</v>
       </c>
       <c r="D38" s="7" t="n">
-        <v>4.851079136958488</v>
+        <v>4.745874305379804</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>4.466417745378932</v>
+        <v>4.361212913800246</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>4.081756353799374</v>
+        <v>3.97655152222069</v>
       </c>
     </row>
     <row r="40">
@@ -3344,19 +3344,19 @@
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>4.851079136958488</v>
+        <v>4.745874305379804</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>5.105682872488786</v>
+        <v>5.0004780409101</v>
       </c>
       <c r="D42" s="7" t="n">
-        <v>5.272987469829767</v>
+        <v>5.167782638251081</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>5.398465917835503</v>
+        <v>5.293261086256817</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>5.607596664511728</v>
+        <v>5.502391832933043</v>
       </c>
     </row>
     <row r="44">
@@ -3401,19 +3401,19 @@
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>4.666619172766612</v>
+        <v>4.562468056436314</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>4.758849154862552</v>
+        <v>4.654171180908059</v>
       </c>
       <c r="D46" s="7" t="n">
-        <v>4.851079136958488</v>
+        <v>4.745874305379804</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>4.943309119054425</v>
+        <v>4.837577429851549</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>5.035539101150361</v>
+        <v>4.929280554323295</v>
       </c>
     </row>
     <row r="48">
@@ -3496,7 +3496,7 @@
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>2.750417615655593</v>
+        <v>2.687145695130762</v>
       </c>
     </row>
     <row r="51">
@@ -3530,7 +3530,7 @@
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>1.121883543030733</v>
+        <v>1.081007637294689</v>
       </c>
     </row>
     <row r="52">
@@ -3564,7 +3564,7 @@
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>7.044222881257744</v>
+        <v>6.913529127525565</v>
       </c>
     </row>
     <row r="53">
@@ -4117,14 +4117,14 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>1.121883543030733</v>
+        <v>1.081007637294689</v>
       </c>
       <c r="C5" s="8">
         <f>'Fundamental Valuation'!C5</f>
         <v/>
       </c>
       <c r="D5" s="7" t="n">
-        <v>7.044222881257744</v>
+        <v>6.913529127525565</v>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
@@ -4291,7 +4291,7 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>2.750417615655593</v>
+        <v>2.687145695130762</v>
       </c>
       <c r="G14" s="9">
         <f>C14/$C$16-1</f>
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>2.750417615655593</v>
+        <v>2.687145695130762</v>
       </c>
     </row>
     <row r="15">
@@ -4597,7 +4597,7 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1.121883543030733</v>
+        <v>1.081007637294689</v>
       </c>
     </row>
     <row r="16">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>7.044222881257744</v>
+        <v>6.913529127525565</v>
       </c>
     </row>
     <row r="18">
@@ -8431,11 +8431,11 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Terminal NOPAT (FY2031E)</t>
+          <t>FY2030E NOPAT — the perpetuity grows this once</t>
         </is>
       </c>
       <c r="C50" s="37">
-        <f>F37*(1+Assumptions!$C$50)</f>
+        <f>F37</f>
         <v/>
       </c>
     </row>
@@ -8446,7 +8446,7 @@
         </is>
       </c>
       <c r="C51" s="37">
-        <f>F35*(1+Assumptions!$C$50)</f>
+        <f>F35</f>
         <v/>
       </c>
     </row>
@@ -8479,7 +8479,7 @@
         </is>
       </c>
       <c r="C54" s="37">
-        <f>-Assumptions!$C$49*-7184.461799</f>
+        <f>-Assumptions!$C$49*-7009.244700</f>
         <v/>
       </c>
     </row>

</xml_diff>